<commit_message>
improve 対応記録.xlsx readability (A-1 through A-6 + B-1)
- B-1: fix _shrink_table to snapshot/reconstruct merged cells after
  delete_rows (openpyxl doesn't shift merges on delete, causing
  MergedCell write errors in fill_investigation)
- A-5: extract_section now matches headings with ■/● prefix and
  テーブル/一覧/:suffix; replace truncate fallback with explicit message
- A-2: separate 影響範囲 (affected flows, parsed from bullets) from
  関連コンポーネント (changed components, parsed from table)
- A-4: use file mtime for each timeline phase instead of all-same now()
- A-3: replace （実装時記入）/（実行後） with empty string to reduce
  placeholder clutter in 対応内容 and テスト sheets
- A-6: rename template 名前→対象 (関連コンポーネント), API名→対象
  (リリース対象一覧) for consistent column naming

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/python/backlog-xlsx/対応記録テンプレート.xlsx
+++ b/scripts/python/backlog-xlsx/対応記録テンプレート.xlsx
@@ -907,8 +907,8 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A17:F17"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B13:F13"/>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>名前</t>
+          <t>対象</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>API名</t>
+          <t>対象</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Group K — 残ファイル追加（create_records・planner・README・テンプレ.xlsx）
patch_template_v7.py は前コミットで追加済み。本コミットで残りを補完:
- create_records.py: border 青色統一・5列化・wording 規約対応
- backlog-planner.md: wording 規約刷新（概要60字・メリ/デメ30字・工数20字）
- _README.md: §日本語規約 に方針比較テーブル文字数注記を追加
- 対応記録テンプレート.xlsx: 対応方針シート 5列化適用済み

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/python/backlog-xlsx/対応記録テンプレート.xlsx
+++ b/scripts/python/backlog-xlsx/対応記録テンプレート.xlsx
@@ -1116,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1150,25 +1150,20 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>方針名</t>
+          <t>概要</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>概要</t>
+          <t>メリット</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>メリット</t>
+          <t>デメリット</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>デメリット</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>工数</t>
         </is>
@@ -1180,7 +1175,6 @@
       <c r="C4" s="6" t="n"/>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5" ht="80" customHeight="1">
       <c r="A5" s="9" t="n"/>
@@ -1188,7 +1182,6 @@
       <c r="C5" s="9" t="n"/>
       <c r="D5" s="9" t="n"/>
       <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
     </row>
     <row r="6" ht="8" customHeight="1"/>
     <row r="7" ht="28" customHeight="1">
@@ -1211,40 +1204,32 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>確認内容</t>
-        </is>
-      </c>
+      <c r="B11" s="22" t="n"/>
       <c r="C11" s="21" t="n"/>
       <c r="D11" s="21" t="n"/>
-      <c r="E11" s="21" t="n"/>
-      <c r="F11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="35" t="n"/>
-      <c r="B12" s="36" t="n"/>
-      <c r="C12" s="35" t="inlineStr"/>
-      <c r="D12" s="36" t="inlineStr"/>
+      <c r="B12" s="35" t="inlineStr"/>
+      <c r="C12" s="36" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="35" t="n"/>
-      <c r="B13" s="36" t="n"/>
-      <c r="C13" s="35" t="inlineStr"/>
-      <c r="D13" s="36" t="inlineStr"/>
+      <c r="B13" s="35" t="inlineStr"/>
+      <c r="C13" s="36" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="35" t="n"/>
-      <c r="B14" s="36" t="n"/>
-      <c r="C14" s="35" t="inlineStr"/>
-      <c r="D14" s="36" t="inlineStr"/>
+      <c r="B14" s="35" t="inlineStr"/>
+      <c r="C14" s="36" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="35" t="n"/>
-      <c r="B15" s="36" t="n"/>
-      <c r="C15" s="35" t="inlineStr"/>
-      <c r="D15" s="36" t="inlineStr"/>
-    </row>
+      <c r="B15" s="35" t="inlineStr"/>
+      <c r="C15" s="36" t="inlineStr"/>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
@@ -1273,16 +1258,16 @@
     <row r="30" ht="35" customHeight="1"/>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9"/>
@@ -1878,7 +1863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2009,18 +1994,18 @@
   <mergeCells count="15">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A9:D9"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Group O: テスト責務二分化（ClaudeCode 自動 vs UI 手動）+ Playwright 廃止
- 対応記録「テスト・検証」シートに ClaudeCode 自動実行テストのみを記載。
  実行種別（Apex Test/SOQL/CLI/メタデータ確認/ファイル確認）列を C 列に追加し 8 列化。
  UI手動行はフィルタして対応記録に載せず、エビデンス.xlsx 側で人が管理する。
- Playwright MCP を全廃。backlog-tester §4 を「ClaudeCode 自動テスト網羅実行」に置き換え。
- create_records.py fill_test: 実行種別 != UI手動 行のみ書き込み・max_col=8。
- create_evidence.py / v2: 実行種別=UI手動 行のみエビデンス側に振り分け。
- backlog-validator Step 6: col 6/7 → col 7/8・UI手動行除外。
- backlog-tester §8①: col 6/7 → col 7/8・UI手動行除外。
- backlog-planner テスト仕様: 実行種別列追加・エビデンス取得方法列廃止・6種ガイド追加。
- _README.md 責務分担表: テスト・検証=自動のみ・エビデンス.xlsx=UI手動（人）に分離。

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/python/backlog-xlsx/対応記録テンプレート.xlsx
+++ b/scripts/python/backlog-xlsx/対応記録テンプレート.xlsx
@@ -1313,7 +1313,6 @@
       <c r="B14" s="35" t="inlineStr"/>
       <c r="C14" s="36" t="inlineStr"/>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
@@ -1343,7 +1342,6 @@
     <row r="30" ht="35" customHeight="1"/>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A7:E7"/>
@@ -1352,6 +1350,7 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9"/>
@@ -1657,12 +1656,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
@@ -1708,25 +1708,30 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
+          <t>実行種別</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
           <t>テスト項目</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>確認方法</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>期待結果</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>実際の結果</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>判定</t>
         </is>
@@ -1742,82 +1747,82 @@
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="6" t="n"/>
       <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="9" t="n"/>
       <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
       <c r="D9" s="9" t="n"/>
       <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="n"/>
       <c r="G9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr"/>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="6" t="n"/>
       <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="9" t="n"/>
       <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="n"/>
       <c r="G11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr"/>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="6" t="n"/>
       <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
       <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="9" t="n"/>
       <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
       <c r="D13" s="9" t="n"/>
       <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="n"/>
       <c r="G13" s="9" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr"/>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="6" t="n"/>
       <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="inlineStr"/>
+      <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
       <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
       <c r="D15" s="9" t="n"/>
       <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="inlineStr"/>
+      <c r="F15" s="9" t="n"/>
       <c r="G15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9"/>

</xml_diff>